<commit_message>
fixed some issues with new companies
</commit_message>
<xml_diff>
--- a/venv/Scripts/job_search_results.xlsx
+++ b/venv/Scripts/job_search_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -623,12 +623,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Software Engineer II - Java</t>
+          <t>Software Engineer II- Java, AWS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210752182</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210742383</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sr Manager of Software Engineering - React framework</t>
+          <t>Software Engineer II - Java</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -670,17 +670,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210753350</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210752182</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Senior Manager of Software Engineering - Java</t>
+          <t>Sr Manager of Software Engineering - React framework</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -707,17 +707,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210757781</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210753350</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Software Engineer II- Java</t>
+          <t>Senior Manager of Software Engineering - Java</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210761687</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210757781</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Software Engineer II - Java, Springboot, Microservices</t>
+          <t>Software Engineer II- Java</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210763350</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210761687</t>
         </is>
       </c>
     </row>
@@ -808,27 +808,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineer II - Java, Springboot, Microservices</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210764822</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210763350</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Software Engineer III</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -855,17 +855,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210765269</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210764822</t>
         </is>
       </c>
     </row>
@@ -882,12 +882,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Software Engineer III - Java Backend, Kafka, AWS, DevOps</t>
+          <t>Software Engineer III</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -897,12 +897,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210771964</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210765269</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Software Engineer II - Devops , Terraform , Kubernetes, Cloud , Python</t>
+          <t>Software Engineer III - Java Backend, Kafka, AWS, DevOps</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210772312</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210771964</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Software Engineer III</t>
+          <t>Software Engineer II - Devops , Terraform , Kubernetes, Cloud , Python</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -966,17 +966,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210776707</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210772312</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Software Engineer II</t>
+          <t>Software Engineer III</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1008,12 +1008,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210777093</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210776707</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Software Engineer III - Data Engineer - Java, Spark, Databricks</t>
+          <t>Software Engineer II</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1040,17 +1040,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778613</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210777093</t>
         </is>
       </c>
     </row>
@@ -1067,17 +1067,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Software Engineer III - Python, PySpark, Databricks, Big Data</t>
+          <t>Software Engineer III - Data Engineer - Java, Spark, Databricks</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778800</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778613</t>
         </is>
       </c>
     </row>
@@ -1099,17 +1099,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Oracle</t>
+          <t>JPMorgan Chase</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Senior Application Software Engineer</t>
+          <t>Software Engineer III - Python, PySpark, Databricks, Big Data</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1119,12 +1119,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/336842</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778800</t>
         </is>
       </c>
     </row>
@@ -1136,32 +1136,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Oracle</t>
+          <t>JPMorgan Chase</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Senior Application Software Engineer</t>
+          <t>Software Engineer III-Java, Kafka/Streams</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BENGALURU, KARNATAKA, India</t>
+          <t>Mumbai, Maharashtra, India</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/337862</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778988</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1178,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Application Software Engineer 2</t>
+          <t>Senior Application Software Engineer</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BENGALURU, KARNATAKA, India</t>
+          <t>India</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1193,12 +1193,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340778</t>
+          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/336842</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Application Software Engineer 2</t>
+          <t>Senior Application Software Engineer</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340777</t>
+          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/337862</t>
         </is>
       </c>
     </row>
@@ -1247,17 +1247,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Oracle</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Application Software Engineer 2</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>BENGALURU, KARNATAKA, India</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1267,12 +1267,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-278536/apply</t>
+          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340778</t>
         </is>
       </c>
     </row>
@@ -1284,17 +1284,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Oracle</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Lead Software Engineer - Agentic Systems</t>
+          <t>Application Software Engineer 2</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>BENGALURU, KARNATAKA, India</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer---Agentic-Systems_R-279158-1/apply</t>
+          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340777</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Software Engineering Manager</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineering-Manager_R-277922-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-278536/apply</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Lead Software Engineer - Agentic Systems</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1378,12 +1378,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-280843/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer---Agentic-Systems_R-279158-1/apply</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineering Manager</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1415,12 +1415,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-287556-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineering-Manager_R-277922-1/apply</t>
         </is>
       </c>
     </row>
@@ -1452,12 +1452,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282489/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-280843/apply</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Lead Software Engineer (Connex)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer--Connex-_R-281114-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-287556-1/apply</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-288230/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282489/apply</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Software Engineer II</t>
+          <t>Lead Software Engineer (Connex)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-281700-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer--Connex-_R-281114-1/apply</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282632/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-288230/apply</t>
         </is>
       </c>
     </row>
@@ -1637,12 +1637,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-287513/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-281700-1/apply</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Lead, Software Engineer</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1674,12 +1674,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead--Software-Engineer_R-287449/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282632/apply</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineer II</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1711,12 +1711,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-280735-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-287513/apply</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Lead, Software Engineer</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1748,12 +1748,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-286411/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead--Software-Engineer_R-287449/apply</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Android</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Vadodara, India</t>
+          <t>Pune, Mahārāshtra, India</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1785,12 +1785,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Vadodara-India/Senior-Software-Engineer---Android_R-274233-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-280735-1/apply</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1822,12 +1822,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282795/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-286411/apply</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1844,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior Software Engineer - Android</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>Vadodara, India</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-281852/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Vadodara-India/Senior-Software-Engineer---Android_R-274233-1/apply</t>
         </is>
       </c>
     </row>
@@ -1876,22 +1876,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PhonePe</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Engineering Manager, Backend</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Pune, Mahārāshtra, India</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/phonepe/jobs/7847265003</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282795/apply</t>
         </is>
       </c>
     </row>
@@ -1913,32 +1913,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Supply Chain Manager II, ROC Reactive Scheduling</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, IND</t>
+          <t>Pune, Mahārāshtra, India</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.amazon.jobs/en/jobs/10499555/supply-chain-manager-ii-roc-reactive-scheduling</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-281852/apply</t>
         </is>
       </c>
     </row>
@@ -1950,32 +1950,32 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>PhonePe</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SDE, International Cobranded Credit Cards</t>
+          <t>Engineering Manager, Backend</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, IND</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.amazon.jobs/en/jobs/10498355/sde-international-cobranded-credit-cards</t>
+          <t>https://job-boards.greenhouse.io/phonepe/jobs/7847265003</t>
         </is>
       </c>
     </row>
@@ -1992,27 +1992,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SysDev I - Multimedia, Amazon Devices</t>
+          <t>Supply Chain Manager II, ROC Reactive Scheduling</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, IND</t>
+          <t>Hyderabad, Telangana, IND</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.amazon.jobs/en/jobs/10501186/sysdev-i-multimedia-amazon-devices</t>
+          <t>https://www.amazon.jobs/en/jobs/10499555/supply-chain-manager-ii-roc-reactive-scheduling</t>
         </is>
       </c>
     </row>
@@ -2024,32 +2024,32 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>SDE, International Cobranded Credit Cards</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>India | Pune, India</t>
+          <t>Bengaluru, Karnataka, IND</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://careers.bp.com/job-description/RQ109868</t>
+          <t>https://www.amazon.jobs/en/jobs/10498355/sde-international-cobranded-credit-cards</t>
         </is>
       </c>
     </row>
@@ -2061,17 +2061,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Security Software Engineer</t>
+          <t>SysDev I - Multimedia, Amazon Devices</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Cohesity - Bangalore - Elnath</t>
+          <t>Chennai, Tamil Nadu, IND</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2081,12 +2081,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Pune---Panchshil---India-Office/Security-Software-Engineer_R03750/apply</t>
+          <t>https://www.amazon.jobs/en/jobs/10501186/sysdev-i-multimedia-amazon-devices</t>
         </is>
       </c>
     </row>
@@ -2098,32 +2098,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>BP</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Senior Manager, Software Engineering</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>India | Pune, India</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Senior-Manager--Software-Engineering_R03690/apply</t>
+          <t>https://careers.bp.com/job-description/RQ109868</t>
         </is>
       </c>
     </row>
@@ -2140,12 +2140,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Security Software Engineer</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>Cohesity - Bangalore - Elnath</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Senior-Software-Engineer_R03151/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Pune---Panchshil---India-Office/Security-Software-Engineer_R03750/apply</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Senior Manager, Software Engineering</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer_R04234/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Senior-Manager--Software-Engineering_R03690/apply</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Software Engineer (C++, Golang, Python)</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer--C----Golang--Python-_R03160/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Senior-Software-Engineer_R03151/apply</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Software Engineer (C/C++, Linux/Windows, Troubleshooting/Debugging)</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer--C-C----Linux-Windows--Troubleshooting-Debugging-_R02047/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer_R04234/apply</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Software Engineer in Test</t>
+          <t>Software Engineer (C++, Golang, Python)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer-in-Test_R03020/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer--C----Golang--Python-_R03160/apply</t>
         </is>
       </c>
     </row>
@@ -2325,12 +2325,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Staff Software Engineer</t>
+          <t>Software Engineer (C/C++, Linux/Windows, Troubleshooting/Debugging)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Cohesity - Bangalore - Elnath</t>
+          <t>Bangalore - India (Office)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Cohesity---Bangalore---Elnath/Software-Engineer--Storage-Filesystem_R02376/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer--C-C----Linux-Windows--Troubleshooting-Debugging-_R02047/apply</t>
         </is>
       </c>
     </row>
@@ -2362,12 +2362,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Staff Software Engineer (Performance Engineering)</t>
+          <t>Software Engineer in Test</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Cohesity - Pune - Panchshil</t>
+          <t>Bangalore - India (Office)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Cohesity---Pune---Panchshil/Staff-Software-Engineer_R02619/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer-in-Test_R03020/apply</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Staff Software Engineer: C++, Distributed Storage, filesystems &amp; cloud skills</t>
+          <t>Staff Software Engineer</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Pune - Panchshil - India (Office)</t>
+          <t>Cohesity - Bangalore - Elnath</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Pune---Panchshil---India-Office/Staff-Software-Engineer--C----Distributed-Storage--filesystems---cloud-skills_R02467/apply</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Cohesity---Bangalore---Elnath/Software-Engineer--Storage-Filesystem_R02376/apply</t>
         </is>
       </c>
     </row>
@@ -2431,22 +2431,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Cohesity</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Java Developer</t>
+          <t>Staff Software Engineer (Performance Engineering)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Cohesity - Pune - Panchshil</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-developer/287/99156611504</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Cohesity---Pune---Panchshil/Staff-Software-Engineer_R02619/apply</t>
         </is>
       </c>
     </row>
@@ -2468,22 +2468,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Cohesity</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Java Middleware Engineer</t>
+          <t>Staff Software Engineer: C++, Distributed Storage, filesystems &amp; cloud skills</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune - Panchshil - India (Office)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-middleware-engineer/287/99123076976</t>
+          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Pune---Panchshil---India-Office/Staff-Software-Engineer--C----Distributed-Storage--filesystems---cloud-skills_R02467/apply</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Java Backend developer</t>
+          <t>Java Developer</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-backend-developer/287/99123076064</t>
+          <t>https://jobs.citi.com/job/pune/java-developer/287/99156611504</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Application Support Analyst - Backend and Data Applications</t>
+          <t>Java Middleware Engineer</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/application-support-analyst-backend-and-data-applications/287/93375538832</t>
+          <t>https://jobs.citi.com/job/pune/java-middleware-engineer/287/99123076976</t>
         </is>
       </c>
     </row>
@@ -2584,17 +2584,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Java Backend</t>
+          <t>Java Backend developer</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239904</t>
+          <t>https://jobs.citi.com/job/pune/java-backend-developer/287/99123076064</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2621,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Java Backend</t>
+          <t>Application Support Analyst - Backend and Data Applications</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239888</t>
+          <t>https://jobs.citi.com/job/pune/application-support-analyst-backend-and-data-applications/287/93375538832</t>
         </is>
       </c>
     </row>
@@ -2658,17 +2658,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Backend Java Blockchain Engineer - Digital Assets Platform</t>
+          <t>Java Backend</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/backend-java-blockchain-engineer-digital-assets-platform/287/98742224064</t>
+          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239904</t>
         </is>
       </c>
     </row>
@@ -2695,17 +2695,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Java Fullstack Angular Developer</t>
+          <t>Java Backend</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-fullstack-angular-developer/287/94439224800</t>
+          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239888</t>
         </is>
       </c>
     </row>
@@ -2732,17 +2732,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Java Full stack Developer</t>
+          <t>Backend Java Blockchain Engineer - Digital Assets Platform</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-java-full-stack-developer/287/98098260048</t>
+          <t>https://jobs.citi.com/job/pune/backend-java-blockchain-engineer-digital-assets-platform/287/98742224064</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Java Full stack Developer</t>
+          <t>Java Fullstack Angular Developer</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-java-full-stack-developer/287/98098260016</t>
+          <t>https://jobs.citi.com/job/pune/java-fullstack-angular-developer/287/94439224800</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Full stack Java React Developer</t>
+          <t>Reactivate Your Career Program – Java Full stack Developer</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316384</t>
+          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-java-full-stack-developer/287/98098260048</t>
         </is>
       </c>
     </row>
@@ -2843,12 +2843,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Full stack Java React Developer</t>
+          <t>Reactivate Your Career Program – Java Full stack Developer</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316368</t>
+          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-java-full-stack-developer/287/98098260016</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Java Microservices Tech lead- Vice President</t>
+          <t>Full stack Java React Developer</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-microservices-tech-lead-vice-president/287/95080353808</t>
+          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316384</t>
         </is>
       </c>
     </row>
@@ -2917,17 +2917,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Public Cloud - Backend Developer Lead – Senior Vice President</t>
+          <t>Full stack Java React Developer</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/public-cloud-backend-developer-lead-senior-vice-president/287/93452215280</t>
+          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316368</t>
         </is>
       </c>
     </row>
@@ -2954,17 +2954,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Full Stack AI Enabled Developer - Java and Angular</t>
+          <t>Java Microservices Tech lead- Vice President</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/full-stack-ai-enabled-developer-java-and-angular/287/97223901072</t>
+          <t>https://jobs.citi.com/job/chennai/java-microservices-tech-lead-vice-president/287/95080353808</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Java Full Stack Engineer</t>
+          <t>Public Cloud - Backend Developer Lead – Senior Vice President</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-full-stack-engineer/287/93375570224</t>
+          <t>https://jobs.citi.com/job/pune/public-cloud-backend-developer-lead-senior-vice-president/287/93452215280</t>
         </is>
       </c>
     </row>
@@ -3028,7 +3028,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Java with React</t>
+          <t>Full Stack AI Enabled Developer - Java and Angular</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-with-react/287/97913195824</t>
+          <t>https://jobs.citi.com/job/pune/full-stack-ai-enabled-developer-java-and-angular/287/97223901072</t>
         </is>
       </c>
     </row>
@@ -3065,17 +3065,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Fullstack Java and React Developer</t>
+          <t>Java Full Stack Engineer</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/fullstack-java-and-react-developer/287/96773695216</t>
+          <t>https://jobs.citi.com/job/chennai/java-full-stack-engineer/287/93375570224</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Java Angular Developer</t>
+          <t>Java with React</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-angular-developer/287/96773693856</t>
+          <t>https://jobs.citi.com/job/pune/java-with-react/287/97913195824</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Java Full Stack Lead - Vice President</t>
+          <t>Fullstack Java and React Developer</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245131040</t>
+          <t>https://jobs.citi.com/job/pune/fullstack-java-and-react-developer/287/96773695216</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Java Full Stack Lead - Vice President</t>
+          <t>Java Angular Developer</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245130992</t>
+          <t>https://jobs.citi.com/job/pune/java-angular-developer/287/96773693856</t>
         </is>
       </c>
     </row>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Java/Python &amp; Flink/Redis Application Development Analyst</t>
+          <t>Java Full Stack Lead - Vice President</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-python-and-flink-redis-application-development-analyst/287/94247930000</t>
+          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245131040</t>
         </is>
       </c>
     </row>
@@ -3250,12 +3250,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Fullstack Java Developer</t>
+          <t>Java Full Stack Lead - Vice President</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599584</t>
+          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245130992</t>
         </is>
       </c>
     </row>
@@ -3287,17 +3287,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Fullstack Java Developer</t>
+          <t>Java/Python &amp; Flink/Redis Application Development Analyst</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599552</t>
+          <t>https://jobs.citi.com/job/pune/java-python-and-flink-redis-application-development-analyst/287/94247930000</t>
         </is>
       </c>
     </row>
@@ -3324,17 +3324,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Java Developer</t>
+          <t>Fullstack Java Developer</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-developer/287/99123076144</t>
+          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599584</t>
         </is>
       </c>
     </row>
@@ -3361,12 +3361,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Senior Java Development Engineer - Vice President</t>
+          <t>Fullstack Java Developer</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/senior-java-development-engineer-vice-president/287/98789768608</t>
+          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599552</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>UI Engineer (Java with React or WPF)</t>
+          <t>Java Developer</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/ui-engineer-java-with-react-or-wpf/287/98836176032</t>
+          <t>https://jobs.citi.com/job/pune/java-developer/287/99123076144</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Java PySpark Bigdata Developer</t>
+          <t>Senior Java Development Engineer - Vice President</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-pyspark-bigdata-developer/287/98789748272</t>
+          <t>https://jobs.citi.com/job/pune/senior-java-development-engineer-vice-president/287/98789768608</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Java Developer with Spark</t>
+          <t>UI Engineer (Java with React or WPF)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-developer-with-spark/287/98789747824</t>
+          <t>https://jobs.citi.com/job/pune/ui-engineer-java-with-react-or-wpf/287/98836176032</t>
         </is>
       </c>
     </row>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Senior Java Technology Lead - Vice President</t>
+          <t>Java PySpark Bigdata Developer</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/senior-java-technology-lead-vice-president/287/95337882480</t>
+          <t>https://jobs.citi.com/job/pune/java-pyspark-bigdata-developer/287/98789748272</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Generative AI Senior Engineer (Python/Java) – Vice President</t>
+          <t>Java Developer with Spark</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/generative-ai-senior-engineer-python-java-vice-president/287/94960988592</t>
+          <t>https://jobs.citi.com/job/pune/java-developer-with-spark/287/98789747824</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Senior Software Engineer Rust OR C++ Equities</t>
+          <t>Senior Java Technology Lead - Vice President</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/senior-software-engineer-rust-or-c-equities/287/98562571728</t>
+          <t>https://jobs.citi.com/job/pune/senior-java-technology-lead-vice-president/287/95337882480</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Python Developer</t>
+          <t>Generative AI Senior Engineer (Python/Java) – Vice President</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-python-developer/287/98098260144</t>
+          <t>https://jobs.citi.com/job/pune/generative-ai-senior-engineer-python-java-vice-president/287/94960988592</t>
         </is>
       </c>
     </row>
@@ -3657,17 +3657,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Python Developer</t>
+          <t>Senior Software Engineer Rust OR C++ Equities</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-python-developer/287/98098260096</t>
+          <t>https://jobs.citi.com/job/pune/senior-software-engineer-rust-or-c-equities/287/98562571728</t>
         </is>
       </c>
     </row>
@@ -3689,32 +3689,217 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>Citi</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Reactivate Your Career Program – Python Developer</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>4+ yrs</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-python-developer/287/98098260144</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Citi</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Reactivate Your Career Program – Python Developer</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu, India</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>4+ yrs</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-python-developer/287/98098260096</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
           <t>Nutanix</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>SDET - Python Automation [ 2 - 4 years ]</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>Bangalore, India</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>2+ yrs</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
         <is>
           <t>https://careers.nutanix.com/en/jobs/32219/sdet-python-automation-2-4-years/</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Software Engineer - SharePoint - Hyderabad</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2+ yrs</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-DTLL-CoRe-DDAI-Application-Development-Analyst/351503</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Software Engineer I/II -  .Net with API Integration + Gen AI - Hyderabad</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2+ yrs</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-Tax-GESTC-Net-API-Integration-Gen-AI-L25-BTA-Hyderabad/353686</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>UK DTS-  Tax -Software Engineer consultant  II- Hyderabad</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2+ yrs</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-UK-DTS-L-35-Tax-Software-Engineer-consultant-II-Hyderabad/356926</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Scheduler file, folder Structure
</commit_message>
<xml_diff>
--- a/venv/Scripts/job_search_results.xlsx
+++ b/venv/Scripts/job_search_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -465,7 +465,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -502,44 +502,44 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Software Engineer II - Java</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2+ yrs</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>JPMorgan Chase</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Software Engineer II</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2+ yrs</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210729807</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210752182</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -549,34 +549,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Software Engineer III - Salesforce Testing</t>
+          <t>Sr Manager of Software Engineering - React framework</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210729978</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210753350</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Software Engineer III - Java/AWS</t>
+          <t>Software Engineer III</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -601,19 +601,19 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210738381</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210765269</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -623,34 +623,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Software Engineer II- Java, AWS</t>
+          <t>Software Engineer III - Java Backend, Kafka, AWS, DevOps</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210742383</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210771964</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Software Engineer II - Java</t>
+          <t>Software Engineer II - Devops , Terraform , Kubernetes, Cloud , Python</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -675,56 +675,56 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210752182</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210772312</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Software Engineer III - Java and Kafka</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3+ yrs</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>JPMorgan Chase</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Sr Manager of Software Engineering - React framework</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210753350</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210775756</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Senior Manager of Software Engineering - Java</t>
+          <t>Software Engineer III</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210757781</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210776707</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Software Engineer II- Java</t>
+          <t>Software Engineer III - Data Engineer - Java, Spark, Databricks</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -791,14 +791,14 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210761687</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778613</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -808,17 +808,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Software Engineer II - Java, Springboot, Microservices</t>
+          <t>Software Engineer III - Python, PySpark, Databricks, Big Data</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -828,14 +828,14 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210763350</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778800</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineer III - Salesforce Testing</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -865,14 +865,14 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210764822</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210729978</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -882,34 +882,34 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Software Engineer III</t>
+          <t>Senior Manager of Software Engineering - Java</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210765269</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210757781</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -919,34 +919,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Software Engineer III - Java Backend, Kafka, AWS, DevOps</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210771964</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210764822</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Software Engineer II - Devops , Terraform , Kubernetes, Cloud , Python</t>
+          <t>Software Engineer II</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -966,76 +966,76 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210772312</t>
+          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210777093</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Senior Application Software Engineer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>JPMorgan Chase</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Software Engineer III</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210776707</t>
+          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/336842</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JPMorgan Chase</t>
+          <t>Oracle</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Software Engineer II</t>
+          <t>Application Software Engineer 2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>BENGALURU, KARNATAKA, India</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1045,71 +1045,71 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210777093</t>
+          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340778</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>JPMorgan Chase</t>
+          <t>Oracle</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Software Engineer III - Data Engineer - Java, Spark, Databricks</t>
+          <t>Application Software Engineer 2</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>BENGALURU, KARNATAKA, India</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778613</t>
+          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340777</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>JPMorgan Chase</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Software Engineer III - Python, PySpark, Databricks, Big Data</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune, Mahārāshtra, India</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1124,140 +1124,140 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778800</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-278536/apply</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>JPMorgan Chase</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Software Engineer III-Java, Kafka/Streams</t>
+          <t>Software Engineering Manager</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra, India</t>
+          <t>Pune, Mahārāshtra, India</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://jpmc.fa.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/210778988</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineering-Manager_R-277922-1/apply</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Software Engineer ||</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pune, Mahārāshtra, India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Oracle</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Senior Application Software Engineer</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/336842</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer---_R-287018/apply</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Pune, Mahārāshtra, India</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Oracle</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Senior Application Software Engineer</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>BENGALURU, KARNATAKA, India</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/337862</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-286526/apply</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Oracle</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Application Software Engineer 2</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BENGALURU, KARNATAKA, India</t>
+          <t>Pune, Mahārāshtra, India</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1267,34 +1267,34 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340778</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-287556-1/apply</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Oracle</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Application Software Engineer 2</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>BENGALURU, KARNATAKA, India</t>
+          <t>Pune, Mahārāshtra, India</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1309,14 +1309,14 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://careers.oracle.com/hcmUI/CandidateExperience/en/sites/jobsearch/job/340777</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282489/apply</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Lead Software Engineer (Connex)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1341,56 +1341,56 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-278536/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer--Connex-_R-281114-1/apply</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Lead Software Engineer</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pune, Mahārāshtra, India</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Lead Software Engineer - Agentic Systems</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Pune, Mahārāshtra, India</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer---Agentic-Systems_R-279158-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-288100/apply</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Software Engineering Manager</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1415,56 +1415,56 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineering-Manager_R-277922-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-288230/apply</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Software Engineer II (Mainframe Developer)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Pune, Mahārāshtra, India</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Lead Software Engineer</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Pune, Mahārāshtra, India</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-280843/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II--Mainframe-Developer-_R-274163/apply</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineer II</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1494,88 +1494,88 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-287556-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-281700-1/apply</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Lead Software Engineer</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Navi Mumbai, India</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Lead Software Engineer</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Pune, Mahārāshtra, India</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282489/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Navi-Mumbai-India-Finicity/Lead-Software-Engineer_R-284367/apply</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Manager, Software Engineering</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Pune, Mahārāshtra, India</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Lead Software Engineer (Connex)</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Pune, Mahārāshtra, India</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer--Connex-_R-281114-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Manager--Software-Engineering_R-281531/apply</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Software Engineer II</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1600,19 +1600,19 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-288230/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-287513/apply</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Software Engineer II</t>
+          <t>Lead, Software Engineer</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1637,56 +1637,56 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-281700-1/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead--Software-Engineer_R-287449/apply</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Pune, Mahārāshtra, India</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Unknown - verify</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Lead Software Engineer</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Pune, Mahārāshtra, India</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Unknown - verify</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282632/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-286411/apply</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Software Engineer II</t>
+          <t>Manager, Software Engineering</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Software-Engineer-II_R-287513/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Manager--Software-Engineering_R-282706/apply</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1733,12 +1733,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Lead, Software Engineer</t>
+          <t>Senior Software Engineer - Android</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>Vadodara, India</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1748,108 +1748,108 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead--Software-Engineer_R-287449/apply</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Vadodara-India/Senior-Software-Engineer---Android_R-274233-1/apply</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Supply Chain Manager II, ROC Reactive Scheduling</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>Hyderabad, Telangana, IND</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-280735-1/apply</t>
+          <t>https://www.amazon.jobs/en/jobs/10499555/supply-chain-manager-ii-roc-reactive-scheduling</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>SDE, International Cobranded Credit Cards</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>Bengaluru, Karnataka, IND</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Senior-Software-Engineer_R-286411/apply</t>
+          <t>https://www.amazon.jobs/en/jobs/10498355/sde-international-cobranded-credit-cards</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Android</t>
+          <t>SysDev I - Multimedia, Amazon Devices</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Vadodara, India</t>
+          <t>Chennai, Tamil Nadu, IND</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1864,103 +1864,103 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Vadodara-India/Senior-Software-Engineer---Android_R-274233-1/apply</t>
+          <t>https://www.amazon.jobs/en/jobs/10501186/sysdev-i-multimedia-amazon-devices</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>BP</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>India | Pune, India</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-282795/apply</t>
+          <t>https://careers.bp.com/job-description/RQ109868</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Java Developer</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Pune, Mahārāshtra, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Lead-Software-Engineer_R-281852/apply</t>
+          <t>https://jobs.citi.com/job/pune/java-developer/287/99156611504</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PhonePe</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Engineering Manager, Backend</t>
+          <t>Java Middleware Engineer</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1970,108 +1970,108 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/phonepe/jobs/7847265003</t>
+          <t>https://jobs.citi.com/job/pune/java-middleware-engineer/287/99123076976</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Supply Chain Manager II, ROC Reactive Scheduling</t>
+          <t>Java Backend developer</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, IND</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.amazon.jobs/en/jobs/10499555/supply-chain-manager-ii-roc-reactive-scheduling</t>
+          <t>https://jobs.citi.com/job/pune/java-backend-developer/287/99123076064</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SDE, International Cobranded Credit Cards</t>
+          <t>Application Support Analyst - Backend and Data Applications</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, IND</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.amazon.jobs/en/jobs/10498355/sde-international-cobranded-credit-cards</t>
+          <t>https://jobs.citi.com/job/pune/application-support-analyst-backend-and-data-applications/287/93375538832</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SysDev I - Multimedia, Amazon Devices</t>
+          <t>Java Backend</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, IND</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2081,76 +2081,76 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.amazon.jobs/en/jobs/10501186/sysdev-i-multimedia-amazon-devices</t>
+          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239904</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Java Backend</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>India | Pune, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://careers.bp.com/job-description/RQ109868</t>
+          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239888</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Security Software Engineer</t>
+          <t>Java Fullstack Angular Developer</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Cohesity - Bangalore - Elnath</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2160,34 +2160,34 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Pune---Panchshil---India-Office/Security-Software-Engineer_R03750/apply</t>
+          <t>https://jobs.citi.com/job/pune/java-fullstack-angular-developer/287/94439224800</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Senior Manager, Software Engineering</t>
+          <t>Reactivate Your Career Program – Java Full stack Developer</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2197,34 +2197,34 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Senior-Manager--Software-Engineering_R03690/apply</t>
+          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-java-full-stack-developer/287/98098260048</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Reactivate Your Career Program – Java Full stack Developer</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2234,34 +2234,34 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Senior-Software-Engineer_R03151/apply</t>
+          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-java-full-stack-developer/287/98098260016</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Full stack Java React Developer</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2271,34 +2271,34 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer_R04234/apply</t>
+          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316384</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Software Engineer (C++, Golang, Python)</t>
+          <t>Full stack Java React Developer</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2308,29 +2308,29 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer--C----Golang--Python-_R03160/apply</t>
+          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316368</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Software Engineer (C/C++, Linux/Windows, Troubleshooting/Debugging)</t>
+          <t>Java Microservices Tech lead- Vice President</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2345,29 +2345,29 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer--C-C----Linux-Windows--Troubleshooting-Debugging-_R02047/apply</t>
+          <t>https://jobs.citi.com/job/chennai/java-microservices-tech-lead-vice-president/287/95080353808</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Software Engineer in Test</t>
+          <t>Public Cloud - Backend Developer Lead – Senior Vice President</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Bangalore - India (Office)</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2382,34 +2382,34 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Bangalore---India-Office/Software-Engineer-in-Test_R03020/apply</t>
+          <t>https://jobs.citi.com/job/pune/public-cloud-backend-developer-lead-senior-vice-president/287/93452215280</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Staff Software Engineer</t>
+          <t>Full Stack AI Enabled Developer - Java and Angular</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Cohesity - Bangalore - Elnath</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2419,34 +2419,34 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Cohesity---Bangalore---Elnath/Software-Engineer--Storage-Filesystem_R02376/apply</t>
+          <t>https://jobs.citi.com/job/pune/full-stack-ai-enabled-developer-java-and-angular/287/97223901072</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Staff Software Engineer (Performance Engineering)</t>
+          <t>Java Full Stack Engineer</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Cohesity - Pune - Panchshil</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2456,34 +2456,34 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Cohesity---Pune---Panchshil/Staff-Software-Engineer_R02619/apply</t>
+          <t>https://jobs.citi.com/job/chennai/java-full-stack-engineer/287/93375570224</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Staff Software Engineer: C++, Distributed Storage, filesystems &amp; cloud skills</t>
+          <t>Java with React</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Pune - Panchshil - India (Office)</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2493,14 +2493,14 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://cohesity.wd5.myworkdayjobs.com/Cohesity_Careers/job/Pune---Panchshil---India-Office/Staff-Software-Engineer--C----Distributed-Storage--filesystems---cloud-skills_R02467/apply</t>
+          <t>https://jobs.citi.com/job/pune/java-with-react/287/97913195824</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Java Developer</t>
+          <t>Fullstack Java and React Developer</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2530,14 +2530,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-developer/287/99156611504</t>
+          <t>https://jobs.citi.com/job/pune/fullstack-java-and-react-developer/287/96773695216</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Java Middleware Engineer</t>
+          <t>Java Angular Developer</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2567,14 +2567,14 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-middleware-engineer/287/99123076976</t>
+          <t>https://jobs.citi.com/job/pune/java-angular-developer/287/96773693856</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Java Backend developer</t>
+          <t>Java Full Stack Lead - Vice President</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2604,14 +2604,14 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-backend-developer/287/99123076064</t>
+          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245131040</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Application Support Analyst - Backend and Data Applications</t>
+          <t>Java Full Stack Lead - Vice President</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2641,14 +2641,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/application-support-analyst-backend-and-data-applications/287/93375538832</t>
+          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245130992</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2658,17 +2658,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Java Backend</t>
+          <t>Java/Python &amp; Flink/Redis Application Development Analyst</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2678,14 +2678,14 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239904</t>
+          <t>https://jobs.citi.com/job/pune/java-python-and-flink-redis-application-development-analyst/287/94247930000</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Java Backend</t>
+          <t>Fullstack Java Developer</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2715,14 +2715,14 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-backend/287/97466239888</t>
+          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599584</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2732,17 +2732,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Backend Java Blockchain Engineer - Digital Assets Platform</t>
+          <t>Fullstack Java Developer</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2752,14 +2752,14 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/backend-java-blockchain-engineer-digital-assets-platform/287/98742224064</t>
+          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599552</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Java Fullstack Angular Developer</t>
+          <t>Java Developer</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2789,14 +2789,14 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-fullstack-angular-developer/287/94439224800</t>
+          <t>https://jobs.citi.com/job/pune/java-developer/287/99123076144</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2806,17 +2806,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Java Full stack Developer</t>
+          <t>Senior Java Development Engineer - Vice President</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2826,14 +2826,14 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-java-full-stack-developer/287/98098260048</t>
+          <t>https://jobs.citi.com/job/pune/senior-java-development-engineer-vice-president/287/98789768608</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Java Full stack Developer</t>
+          <t>UI Engineer (Java with React or WPF)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2863,14 +2863,14 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-java-full-stack-developer/287/98098260016</t>
+          <t>https://jobs.citi.com/job/pune/ui-engineer-java-with-react-or-wpf/287/98836176032</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2880,12 +2880,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Full stack Java React Developer</t>
+          <t>Java PySpark Bigdata Developer</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2900,14 +2900,14 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316384</t>
+          <t>https://jobs.citi.com/job/pune/java-pyspark-bigdata-developer/287/98789748272</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2917,12 +2917,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Full stack Java React Developer</t>
+          <t>Java Developer with Spark</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2937,14 +2937,14 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/full-stack-java-react-developer/287/97603316368</t>
+          <t>https://jobs.citi.com/job/pune/java-developer-with-spark/287/98789747824</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2954,17 +2954,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Java Microservices Tech lead- Vice President</t>
+          <t>Senior Java Technology Lead - Vice President</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>3+ yrs</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -2974,14 +2974,14 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-microservices-tech-lead-vice-president/287/95080353808</t>
+          <t>https://jobs.citi.com/job/pune/senior-java-technology-lead-vice-president/287/95337882480</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Public Cloud - Backend Developer Lead – Senior Vice President</t>
+          <t>Generative AI Senior Engineer (Python/Java) – Vice President</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3011,14 +3011,14 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/public-cloud-backend-developer-lead-senior-vice-president/287/93452215280</t>
+          <t>https://jobs.citi.com/job/pune/generative-ai-senior-engineer-python-java-vice-president/287/94960988592</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Full Stack AI Enabled Developer - Java and Angular</t>
+          <t>Senior Software Engineer Rust OR C++ Equities</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3048,14 +3048,14 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/full-stack-ai-enabled-developer-java-and-angular/287/97223901072</t>
+          <t>https://jobs.citi.com/job/pune/senior-software-engineer-rust-or-c-equities/287/98562571728</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3065,17 +3065,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Java Full Stack Engineer</t>
+          <t>Reactivate Your Career Program – Python Developer</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2+ yrs</t>
+          <t>4+ yrs</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3085,14 +3085,14 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/java-full-stack-engineer/287/93375570224</t>
+          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-python-developer/287/98098260144</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3102,12 +3102,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Java with React</t>
+          <t>Reactivate Your Career Program – Python Developer</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3122,103 +3122,103 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-with-react/287/97913195824</t>
+          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-python-developer/287/98098260096</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Fullstack Java and React Developer</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/fullstack-java-and-react-developer/287/96773695216</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer/13015/88422582704</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Java Angular Developer</t>
+          <t>Software Engineer - Full Stack</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-angular-developer/287/96773693856</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer-full-stack/13015/99153508992</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Java Full Stack Lead - Vice President</t>
+          <t>Java Developer</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3228,34 +3228,34 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245131040</t>
+          <t>https://search.jobs.barclays/job/pune/java-developer/13015/97128373024</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Java Full Stack Lead - Vice President</t>
+          <t>Full Stack Developer - VP</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3265,71 +3265,71 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-full-stack-lead-vice-president/287/95245130992</t>
+          <t>https://search.jobs.barclays/job/pune/full-stack-developer-vp/13015/94778649776</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Java/Python &amp; Flink/Redis Application Development Analyst</t>
+          <t>Full Stack Engineer</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-python-and-flink-redis-application-development-analyst/287/94247930000</t>
+          <t>https://search.jobs.barclays/job/pune/full-stack-engineer/13015/99119337632</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Fullstack Java Developer</t>
+          <t>Software Engineer - Android</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3339,34 +3339,34 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599584</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer-android/13015/99203717008</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Fullstack Java Developer</t>
+          <t>Software Engineer - Java</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3376,71 +3376,71 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/chennai/fullstack-java-developer/287/99156599552</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer-java/13015/99203716784</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Java Developer</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-developer/287/99123076144</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer/13015/94687913696</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Senior Java Development Engineer - Vice President</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3450,187 +3450,187 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/senior-java-development-engineer-vice-president/287/98789768608</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer/13015/98800934752</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>UI Engineer (Java with React or WPF)</t>
+          <t>Lead Software Engineer - VP</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/ui-engineer-java-with-react-or-wpf/287/98836176032</t>
+          <t>https://search.jobs.barclays/job/pune/lead-software-engineer-vp/13015/99119343632</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Java PySpark Bigdata Developer</t>
+          <t>Software Engineer​</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-pyspark-bigdata-developer/287/98789748272</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer/13015/99203724880</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Java Developer with Spark</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/java-developer-with-spark/287/98789747824</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer/13015/99203724848</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Senior Java Technology Lead - Vice President</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>3+ yrs</t>
+          <t>Unknown - verify</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/senior-java-technology-lead-vice-president/287/95337882480</t>
+          <t>https://search.jobs.barclays/job/pune/software-engineer/13015/99172224512</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Nutanix</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Generative AI Senior Engineer (Python/Java) – Vice President</t>
+          <t>SDET - Python Automation [ 2 - 4 years ]</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Bangalore, India</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3640,34 +3640,34 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/generative-ai-senior-engineer-python-java-vice-president/287/94960988592</t>
+          <t>https://careers.nutanix.com/en/jobs/32219/sdet-python-automation-2-4-years/</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Senior Software Engineer Rust OR C++ Equities</t>
+          <t>Software Engineer - SharePoint - Hyderabad</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Unknown - verify</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3677,34 +3677,34 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/senior-software-engineer-rust-or-c-equities/287/98562571728</t>
+          <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-DTLL-CoRe-DDAI-Application-Development-Analyst/351503</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Python Developer</t>
+          <t>Software Engineer I/II -  .Net with API Integration + Gen AI - Hyderabad</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3714,34 +3714,34 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/pune/reactivate-your-career-program-python-developer/287/98098260144</t>
+          <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-Tax-GESTC-Net-API-Integration-Gen-AI-L25-BTA-Hyderabad/353686</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Reactivate Your Career Program – Python Developer</t>
+          <t>UK DTS-  Tax -Software Engineer consultant  II- Hyderabad</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>4+ yrs</t>
+          <t>2+ yrs</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3750,154 +3750,6 @@
         </is>
       </c>
       <c r="G90" t="inlineStr">
-        <is>
-          <t>https://jobs.citi.com/job/chennai/reactivate-your-career-program-python-developer/287/98098260096</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Nutanix</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>SDET - Python Automation [ 2 - 4 years ]</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Bangalore, India</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>2+ yrs</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>https://careers.nutanix.com/en/jobs/32219/sdet-python-automation-2-4-years/</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Deloitte</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Software Engineer - SharePoint - Hyderabad</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>2+ yrs</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-DTLL-CoRe-DDAI-Application-Development-Analyst/351503</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Deloitte</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Software Engineer I/II -  .Net with API Integration + Gen AI - Hyderabad</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>2+ yrs</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-Tax-GESTC-Net-API-Integration-Gen-AI-L25-BTA-Hyderabad/353686</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Deloitte</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>UK DTS-  Tax -Software Engineer consultant  II- Hyderabad</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>2+ yrs</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
         <is>
           <t>https://usijobs.deloitte.com/en_US/careersUSI/JobDetail/USI-EH27-UK-DTS-L-35-Tax-Software-Engineer-consultant-II-Hyderabad/356926</t>
         </is>

</xml_diff>